<commit_message>
Daily follower scan: 2026-08-19
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,14 +446,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>nasa</t>
+          <t>indosat</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>104399390</v>
+        <v>1912024</v>
       </c>
       <c r="C2" t="n">
-        <v>104399390</v>
+        <v>1912024</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -465,14 +465,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>natgeo</t>
+          <t>myxl</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>268753774</v>
+        <v>407022</v>
       </c>
       <c r="C3" t="n">
-        <v>268753774</v>
+        <v>407022</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -484,19 +484,76 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>nasa</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>104399390</v>
+      </c>
+      <c r="C4" t="n">
+        <v>104399390</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>natgeo</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>268753774</v>
+      </c>
+      <c r="C5" t="n">
+        <v>268753774</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>nike</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B6" t="n">
         <v>291458025</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C6" t="n">
         <v>291458025</v>
       </c>
-      <c r="D4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" t="n">
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>telkomsel</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>2496940</v>
+      </c>
+      <c r="C7" t="n">
+        <v>2496940</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily follower scan: 2026-08-20
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,58 +446,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>indosat</t>
+          <t>myxl</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1912024</v>
+        <v>407174</v>
       </c>
       <c r="C2" t="n">
-        <v>1912024</v>
+        <v>407022</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>152</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>0.0373</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>myxl</t>
+          <t>telkomsel</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>407022</v>
+        <v>2496936</v>
       </c>
       <c r="C3" t="n">
-        <v>407022</v>
+        <v>2496940</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>telkomsel</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>2496940</v>
-      </c>
-      <c r="C4" t="n">
-        <v>2496940</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0</v>
+        <v>-0.0002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-08-21
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>407443</v>
+      </c>
+      <c r="C2" t="n">
         <v>407174</v>
       </c>
-      <c r="C2" t="n">
-        <v>407022</v>
-      </c>
       <c r="D2" t="n">
-        <v>152</v>
+        <v>269</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0373</v>
+        <v>0.06610000000000001</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2497010</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496936</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496940</v>
-      </c>
       <c r="D3" t="n">
-        <v>-4</v>
+        <v>74</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0002</v>
+        <v>0.003</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-08-22
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>407574</v>
+      </c>
+      <c r="C2" t="n">
         <v>407443</v>
       </c>
-      <c r="C2" t="n">
-        <v>407174</v>
-      </c>
       <c r="D2" t="n">
-        <v>269</v>
+        <v>131</v>
       </c>
       <c r="E2" t="n">
-        <v>0.06610000000000001</v>
+        <v>0.0322</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2497073</v>
+      </c>
+      <c r="C3" t="n">
         <v>2497010</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496936</v>
-      </c>
       <c r="D3" t="n">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="E3" t="n">
-        <v>0.003</v>
+        <v>0.0025</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-08-23
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>407676</v>
+      </c>
+      <c r="C2" t="n">
         <v>407574</v>
       </c>
-      <c r="C2" t="n">
-        <v>407443</v>
-      </c>
       <c r="D2" t="n">
-        <v>131</v>
+        <v>102</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0322</v>
+        <v>0.025</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2497046</v>
+      </c>
+      <c r="C3" t="n">
         <v>2497073</v>
       </c>
-      <c r="C3" t="n">
-        <v>2497010</v>
-      </c>
       <c r="D3" t="n">
-        <v>63</v>
+        <v>-27</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0025</v>
+        <v>-0.0011</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-08-24
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>407770</v>
+      </c>
+      <c r="C2" t="n">
         <v>407676</v>
       </c>
-      <c r="C2" t="n">
-        <v>407574</v>
-      </c>
       <c r="D2" t="n">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="E2" t="n">
-        <v>0.025</v>
+        <v>0.0231</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496965</v>
+      </c>
+      <c r="C3" t="n">
         <v>2497046</v>
       </c>
-      <c r="C3" t="n">
-        <v>2497073</v>
-      </c>
       <c r="D3" t="n">
-        <v>-27</v>
+        <v>-81</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0011</v>
+        <v>-0.0032</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-08-25
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>407897</v>
+      </c>
+      <c r="C2" t="n">
         <v>407770</v>
       </c>
-      <c r="C2" t="n">
-        <v>407676</v>
-      </c>
       <c r="D2" t="n">
-        <v>94</v>
+        <v>127</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0231</v>
+        <v>0.0311</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2497074</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496965</v>
       </c>
-      <c r="C3" t="n">
-        <v>2497046</v>
-      </c>
       <c r="D3" t="n">
-        <v>-81</v>
+        <v>109</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0032</v>
+        <v>0.0044</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-08-26
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>408016</v>
+      </c>
+      <c r="C2" t="n">
         <v>407897</v>
       </c>
-      <c r="C2" t="n">
-        <v>407770</v>
-      </c>
       <c r="D2" t="n">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0311</v>
+        <v>0.0292</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2497100</v>
+      </c>
+      <c r="C3" t="n">
         <v>2497074</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496965</v>
-      </c>
       <c r="D3" t="n">
-        <v>109</v>
+        <v>26</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0044</v>
+        <v>0.001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-08-27
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>408138</v>
+      </c>
+      <c r="C2" t="n">
         <v>408016</v>
       </c>
-      <c r="C2" t="n">
-        <v>407897</v>
-      </c>
       <c r="D2" t="n">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0292</v>
+        <v>0.0299</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2497135</v>
+      </c>
+      <c r="C3" t="n">
         <v>2497100</v>
       </c>
-      <c r="C3" t="n">
-        <v>2497074</v>
-      </c>
       <c r="D3" t="n">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="E3" t="n">
-        <v>0.001</v>
+        <v>0.0014</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-08-28
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>408238</v>
+      </c>
+      <c r="C2" t="n">
         <v>408138</v>
       </c>
-      <c r="C2" t="n">
-        <v>408016</v>
-      </c>
       <c r="D2" t="n">
-        <v>122</v>
+        <v>100</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0299</v>
+        <v>0.0245</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2497181</v>
+      </c>
+      <c r="C3" t="n">
         <v>2497135</v>
       </c>
-      <c r="C3" t="n">
-        <v>2497100</v>
-      </c>
       <c r="D3" t="n">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0014</v>
+        <v>0.0018</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-08-29
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>408300</v>
+      </c>
+      <c r="C2" t="n">
         <v>408238</v>
       </c>
-      <c r="C2" t="n">
-        <v>408138</v>
-      </c>
       <c r="D2" t="n">
-        <v>100</v>
+        <v>62</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0245</v>
+        <v>0.0152</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2497144</v>
+      </c>
+      <c r="C3" t="n">
         <v>2497181</v>
       </c>
-      <c r="C3" t="n">
-        <v>2497135</v>
-      </c>
       <c r="D3" t="n">
-        <v>46</v>
+        <v>-37</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0018</v>
+        <v>-0.0015</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-08-30
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -446,39 +446,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>myxl</t>
+          <t>telkomsel</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>408300</v>
+        <v>2497051</v>
       </c>
       <c r="C2" t="n">
-        <v>408238</v>
+        <v>2497144</v>
       </c>
       <c r="D2" t="n">
-        <v>62</v>
+        <v>-93</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0152</v>
+        <v>-0.0037</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>telkomsel</t>
+          <t>myxl</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2497144</v>
+        <v>408377</v>
       </c>
       <c r="C3" t="n">
-        <v>2497181</v>
+        <v>408300</v>
       </c>
       <c r="D3" t="n">
-        <v>-37</v>
+        <v>77</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0015</v>
+        <v>0.0189</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-08-31
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -446,39 +446,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>telkomsel</t>
+          <t>myxl</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2497051</v>
+        <v>408483</v>
       </c>
       <c r="C2" t="n">
-        <v>2497144</v>
+        <v>408377</v>
       </c>
       <c r="D2" t="n">
-        <v>-93</v>
+        <v>106</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.0037</v>
+        <v>0.026</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>myxl</t>
+          <t>telkomsel</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>408377</v>
+        <v>2496958</v>
       </c>
       <c r="C3" t="n">
-        <v>408300</v>
+        <v>2497051</v>
       </c>
       <c r="D3" t="n">
-        <v>77</v>
+        <v>-93</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0189</v>
+        <v>-0.0037</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-09-01
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>408536</v>
+      </c>
+      <c r="C2" t="n">
         <v>408483</v>
       </c>
-      <c r="C2" t="n">
-        <v>408377</v>
-      </c>
       <c r="D2" t="n">
-        <v>106</v>
+        <v>53</v>
       </c>
       <c r="E2" t="n">
-        <v>0.026</v>
+        <v>0.013</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496936</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496958</v>
       </c>
-      <c r="C3" t="n">
-        <v>2497051</v>
-      </c>
       <c r="D3" t="n">
-        <v>-93</v>
+        <v>-22</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0037</v>
+        <v>-0.0009</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-09-02
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>408595</v>
+      </c>
+      <c r="C2" t="n">
         <v>408536</v>
       </c>
-      <c r="C2" t="n">
-        <v>408483</v>
-      </c>
       <c r="D2" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="E2" t="n">
-        <v>0.013</v>
+        <v>0.0144</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496890</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496936</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496958</v>
-      </c>
       <c r="D3" t="n">
-        <v>-22</v>
+        <v>-46</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0009</v>
+        <v>-0.0018</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-09-03
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -446,39 +446,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>myxl</t>
+          <t>telkomsel</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>408595</v>
+        <v>2496970</v>
       </c>
       <c r="C2" t="n">
-        <v>408536</v>
+        <v>2496890</v>
       </c>
       <c r="D2" t="n">
-        <v>59</v>
+        <v>80</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0144</v>
+        <v>0.0032</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>telkomsel</t>
+          <t>myxl</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2496890</v>
+        <v>408651</v>
       </c>
       <c r="C3" t="n">
-        <v>2496936</v>
+        <v>408595</v>
       </c>
       <c r="D3" t="n">
-        <v>-46</v>
+        <v>56</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0018</v>
+        <v>0.0137</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-09-04
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -446,39 +446,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>telkomsel</t>
+          <t>myxl</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2496970</v>
+        <v>408714</v>
       </c>
       <c r="C2" t="n">
-        <v>2496890</v>
+        <v>408651</v>
       </c>
       <c r="D2" t="n">
-        <v>80</v>
+        <v>63</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0032</v>
+        <v>0.0154</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>myxl</t>
+          <t>telkomsel</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>408651</v>
+        <v>2496991</v>
       </c>
       <c r="C3" t="n">
-        <v>408595</v>
+        <v>2496970</v>
       </c>
       <c r="D3" t="n">
-        <v>56</v>
+        <v>21</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0137</v>
+        <v>0.0008</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-09-05
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>408800</v>
+      </c>
+      <c r="C2" t="n">
         <v>408714</v>
       </c>
-      <c r="C2" t="n">
-        <v>408651</v>
-      </c>
       <c r="D2" t="n">
-        <v>63</v>
+        <v>86</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0154</v>
+        <v>0.021</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496931</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496991</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496970</v>
-      </c>
       <c r="D3" t="n">
-        <v>21</v>
+        <v>-60</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0008</v>
+        <v>-0.0024</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-09-06
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>408901</v>
+      </c>
+      <c r="C2" t="n">
         <v>408800</v>
       </c>
-      <c r="C2" t="n">
-        <v>408714</v>
-      </c>
       <c r="D2" t="n">
-        <v>86</v>
+        <v>101</v>
       </c>
       <c r="E2" t="n">
-        <v>0.021</v>
+        <v>0.0247</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496999</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496931</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496991</v>
-      </c>
       <c r="D3" t="n">
-        <v>-60</v>
+        <v>68</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0024</v>
+        <v>0.0027</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-09-07
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>408996</v>
+      </c>
+      <c r="C2" t="n">
         <v>408901</v>
       </c>
-      <c r="C2" t="n">
-        <v>408800</v>
-      </c>
       <c r="D2" t="n">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0247</v>
+        <v>0.0232</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2497053</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496999</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496931</v>
-      </c>
       <c r="D3" t="n">
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0027</v>
+        <v>0.0022</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-09-08
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -446,39 +446,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>myxl</t>
+          <t>telkomsel</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>408996</v>
+        <v>2496975</v>
       </c>
       <c r="C2" t="n">
-        <v>408901</v>
+        <v>2497053</v>
       </c>
       <c r="D2" t="n">
-        <v>95</v>
+        <v>-78</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0232</v>
+        <v>-0.0031</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>telkomsel</t>
+          <t>myxl</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2497053</v>
+        <v>409058</v>
       </c>
       <c r="C3" t="n">
-        <v>2496999</v>
+        <v>408996</v>
       </c>
       <c r="D3" t="n">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0022</v>
+        <v>0.0152</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-09-09
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -446,39 +446,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>telkomsel</t>
+          <t>myxl</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2496975</v>
+        <v>409158</v>
       </c>
       <c r="C2" t="n">
-        <v>2497053</v>
+        <v>409058</v>
       </c>
       <c r="D2" t="n">
-        <v>-78</v>
+        <v>100</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.0031</v>
+        <v>0.0244</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>myxl</t>
+          <t>telkomsel</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>409058</v>
+        <v>2497018</v>
       </c>
       <c r="C3" t="n">
-        <v>408996</v>
+        <v>2496975</v>
       </c>
       <c r="D3" t="n">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0152</v>
+        <v>0.0017</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-09-10
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -446,39 +446,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>myxl</t>
+          <t>telkomsel</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>409158</v>
+        <v>2496938</v>
       </c>
       <c r="C2" t="n">
-        <v>409058</v>
+        <v>2497018</v>
       </c>
       <c r="D2" t="n">
-        <v>100</v>
+        <v>-80</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0244</v>
+        <v>-0.0032</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>telkomsel</t>
+          <t>myxl</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2497018</v>
+        <v>409228</v>
       </c>
       <c r="C3" t="n">
-        <v>2496975</v>
+        <v>409158</v>
       </c>
       <c r="D3" t="n">
-        <v>43</v>
+        <v>70</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0017</v>
+        <v>0.0171</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-09-11
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -446,39 +446,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>telkomsel</t>
+          <t>myxl</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2496938</v>
+        <v>409373</v>
       </c>
       <c r="C2" t="n">
-        <v>2497018</v>
+        <v>409228</v>
       </c>
       <c r="D2" t="n">
-        <v>-80</v>
+        <v>145</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.0032</v>
+        <v>0.0354</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>myxl</t>
+          <t>telkomsel</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>409228</v>
+        <v>2496994</v>
       </c>
       <c r="C3" t="n">
-        <v>409158</v>
+        <v>2496938</v>
       </c>
       <c r="D3" t="n">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0171</v>
+        <v>0.0022</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-09-12
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -446,39 +446,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>myxl</t>
+          <t>telkomsel</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>409373</v>
+        <v>2496794</v>
       </c>
       <c r="C2" t="n">
-        <v>409228</v>
+        <v>2496994</v>
       </c>
       <c r="D2" t="n">
-        <v>145</v>
+        <v>-200</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0354</v>
+        <v>-0.008</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>telkomsel</t>
+          <t>myxl</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2496994</v>
+        <v>409401</v>
       </c>
       <c r="C3" t="n">
-        <v>2496938</v>
+        <v>409373</v>
       </c>
       <c r="D3" t="n">
-        <v>56</v>
+        <v>28</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0022</v>
+        <v>0.0068</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-09-13
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -446,39 +446,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>telkomsel</t>
+          <t>myxl</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2496794</v>
+        <v>409540</v>
       </c>
       <c r="C2" t="n">
-        <v>2496994</v>
+        <v>409401</v>
       </c>
       <c r="D2" t="n">
-        <v>-200</v>
+        <v>139</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.008</v>
+        <v>0.034</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>myxl</t>
+          <t>telkomsel</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>409401</v>
+        <v>2496824</v>
       </c>
       <c r="C3" t="n">
-        <v>409373</v>
+        <v>2496794</v>
       </c>
       <c r="D3" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0068</v>
+        <v>0.0012</v>
       </c>
     </row>
   </sheetData>

</xml_diff>